<commit_message>
fix: harden noetic_core after the M1 review, think before act in tick, with UT-038 and UT-070 to UT-073
</commit_message>
<xml_diff>
--- a/docs/04_internal_design.xlsx
+++ b/docs/04_internal_design.xlsx
@@ -807,7 +807,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.14</t>
+          <t xml:space="preserve">0.15</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Rust stable, edition 2024, rustfmt default, clippy -D warnings (pedantic for core).</t>
+          <t xml:space="preserve">Rust stable, edition 2024, rustfmt default, clippy -D warnings with the extra lints picked one by one in the workspace [lints]; no clippy::pedantic as a whole.</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>#![forbid(unsafe_code)] in all crates.</t>
+          <t xml:space="preserve">unsafe_code = "forbid" in the workspace [lints], which every crate inherits: the same as #![forbid(unsafe_code)] in each.</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Every pub item has a doc comment with the API ID, e.g. /// API-COR-007 weighted_pick.</t>
+          <t xml:space="preserve">Every pub item that implements a design ID starts its doc comment with that ID, e.g. /// API-COR-007 Picks one item…; helpers that implement none stay pub(crate).</t>
         </is>
       </c>
     </row>
@@ -2593,12 +2593,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>1000 ticks of the default world with seed 42 → hash of agent states equals stored hash.</t>
+          <t xml:space="preserve">1000 ticks of the default world (four rabbits, built in the test) with seed 42 → FNV-1a hash of the world's Debug text equals the GOLDEN constant.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>tests/golden/*.ron</t>
+          <t xml:space="preserve">tests/golden.rs</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3076,6 +3076,28 @@
       <c r="D17" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">TYP-10 names GoToTarget, the target of StepKind::GoTo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.15</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-20</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review of M1: MOD-064 noetic_core::tuning is dropped, every tuning constant is named in the Config section of the file that uses it; TYP-14 is implemented by world::Clock so far and SimWorld never lends itself as a whole, since tick holds its agents mutably: the rest of the world is the view, with positions from the grid built before Think; TST-03 keeps the golden hash as a constant in tests/golden.rs, FNV-1a over the world's Debug text; CS-01 drops clippy::pedantic, since the lints worth having are picked one by one in the workspace [lints]; CS-02 is the workspace lint; CS-04 follows CONTRIBUTING (the design ID starts the doc of the pub items that implement one); the dependency rules are checked by review until the CI exists.</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3502,7 @@
 │  ├─ noetic_core/            # no Bevy dependency
 │  │  └─ src/{lib.rs, model/, agent/, world/, sim.rs, perception.rs, emotion.rs, reaction.rs,
 │  │          utility.rs, steps.rs, social.rs, conflict.rs, territory.rs, locomotion.rs,
-│  │          personality.rs, rng.rs, io/, ext.rs, sandbox.rs, tuning.rs, events.rs}
+│  │          personality.rs, rng.rs, io/, ext.rs, sandbox.rs, events.rs}
 │  ├─ noetic/                 # the crate games add: Bevy plugin, pub use noetic_core, prelude
 │  │  └─ src/{lib.rs, plugin.rs, asset.rs, sync.rs, think.rs, anim.rs, nav.rs, debug.rs}
 │  └─ noetic_editor/          # binary
@@ -5696,7 +5718,7 @@
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Initial tuning constants of the ALG-xx formulas, in one place.</t>
+          <t xml:space="preserve">Dropped (0.15): every tuning constant is named in the Config section of the file that uses it (CONTRIBUTING).</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
@@ -5752,7 +5774,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Enforced in CI (cargo-deny + a test that greps Cargo metadata)</t>
+          <t xml:space="preserve">To be enforced in CI (cargo-deny + a test that greps Cargo metadata); until the CI exists, review checks them.</t>
         </is>
       </c>
     </row>
@@ -6481,7 +6503,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Editor owns one; games use WorldViewCache instead</t>
+          <t xml:space="preserve">Editor owns one; every field but agents and species makes up its WorldView (TYP-14); games use WorldViewCache instead</t>
         </is>
       </c>
     </row>
@@ -6513,7 +6535,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Read-only. Implemented by SimWorld and by noetic::sync::WorldViewCache; per-agent core functions get &amp;dyn WorldView, never the world itself</t>
+          <t xml:space="preserve">Read-only. Implemented by world::Clock while the view asks only hour() and secs_per_game_hour() (M1); SimWorld and noetic::sync::WorldViewCache implement it once it asks more, but never SimWorld as a whole: tick holds its agents mutably, so the view is the rest of the world (the clock now; wind, terrain, marks, stimuli and the grid of positions built before Think later) in a field of its own. Per-agent core functions get &amp;dyn WorldView, never the world itself</t>
         </is>
       </c>
     </row>

</xml_diff>